<commit_message>
Update documentation from internal repository
</commit_message>
<xml_diff>
--- a/doc/source/application/concepts/AHOISpro_RandomProcesses.xlsx
+++ b/doc/source/application/concepts/AHOISpro_RandomProcesses.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IvanDigel\git\ahois-pro\doc\source\_res\application\concepts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IvanDigel\git\ahois-pro\doc\source\application\concepts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50FD833B-2B5E-42EB-AF71-80EC2277733A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{308FA353-3E61-4896-A238-8E84CFB0C5CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -670,7 +670,7 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="1" max="1" width="22.109375" customWidth="1"/>
     <col min="2" max="2" width="28.5546875" customWidth="1"/>
     <col min="3" max="3" width="45.33203125" customWidth="1"/>
     <col min="4" max="4" width="60.88671875" customWidth="1"/>

</xml_diff>